<commit_message>
updat syllabus with room
</commit_message>
<xml_diff>
--- a/00-course-info/S2026/_class-planning-S26.xlsx
+++ b/00-course-info/S2026/_class-planning-S26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cpslo-my.sharepoint.com/personal/erobin17_calpoly_edu/Documents/stat323-calpoly/00-course-info/S2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="514" documentId="13_ncr:1_{3E3E1360-79E0-49B8-888E-E9DF4B34EF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79CEE338-1D28-364F-9DD9-8CD91B2E5733}"/>
+  <xr:revisionPtr revIDLastSave="517" documentId="13_ncr:1_{3E3E1360-79E0-49B8-888E-E9DF4B34EF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{758D7C1E-5C69-C74E-A939-4EFBFD0C1A17}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="162">
   <si>
     <t>Week</t>
   </si>
@@ -499,12 +499,6 @@
     <t>Activity 4.1: Cookie Contrasts</t>
   </si>
   <si>
-    <t>Submit to Canvas by 2/6</t>
-  </si>
-  <si>
-    <t>Submit to Canvas by 1/22</t>
-  </si>
-  <si>
     <t>Activity 5.1: Advertising Strategies</t>
   </si>
   <si>
@@ -539,6 +533,9 @@
   </si>
   <si>
     <t>Project workday</t>
+  </si>
+  <si>
+    <t>Submit to Canvas by 4/15</t>
   </si>
 </sst>
 </file>
@@ -1920,7 +1917,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E2" s="24"/>
       <c r="F2" s="24"/>
@@ -1964,13 +1961,13 @@
         <v>95</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B6" s="28"/>
       <c r="E6" s="25" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>97</v>
@@ -2003,7 +2000,7 @@
         <v>100</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -2111,9 +2108,7 @@
       <c r="F19" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G19" s="15" t="s">
-        <v>149</v>
-      </c>
+      <c r="G19" s="15"/>
     </row>
     <row r="20" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="30">
@@ -2226,7 +2221,7 @@
         <v>124</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
@@ -2286,10 +2281,10 @@
         <v>131</v>
       </c>
       <c r="F39" s="30" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G39" s="30" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2310,7 +2305,7 @@
         <v>132</v>
       </c>
       <c r="F41" s="30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
@@ -2350,10 +2345,10 @@
         <v>135</v>
       </c>
       <c r="F47" s="30" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G47" s="30" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
@@ -2404,7 +2399,7 @@
         <v>3</v>
       </c>
       <c r="D53" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2420,7 +2415,7 @@
         <v>2</v>
       </c>
       <c r="D56" s="30" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2452,7 +2447,7 @@
     <row r="66" spans="4:4" s="30" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="69" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D69" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>